<commit_message>
Add checks for prerequisites in course plan validation
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Frasningskonsistens.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Frasningskonsistens.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Frasningskonsistens" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Frasningskonsistens'!$A$1:$E$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Frasningskonsistens'!$A$1:$E$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -634,7 +634,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BY2025</t>
+          <t>BY3005</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -649,19 +649,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenterna kunna:…</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BY3005</t>
+          <t>GBY2RN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -676,19 +676,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenterna kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RN</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GBY2RN</t>
+          <t>GBY2V5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -708,14 +708,14 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GBY2V5</t>
+          <t>GBY2V8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -730,19 +730,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V8</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GBY2V8</t>
+          <t>GBY33L</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -762,14 +762,14 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY33L</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GBY33L</t>
+          <t>GBY34M</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter godkänd kurs skall den studerande kunna:…</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY33L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34M</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GBY34M</t>
+          <t>GBY34N</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall den studerande kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34N</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GBY34N</t>
+          <t>GBY38D</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -838,19 +838,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY38D</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GBY38D</t>
+          <t>GBY3AX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -865,24 +865,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande för ett konkret husbyggnadsprojekt kunna:…</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY38D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY3AX</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GBY3AX</t>
+          <t>GDT2JM</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>DTA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -892,19 +892,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande för ett konkret husbyggnadsprojekt kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY3AX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JM</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GDT2JM</t>
+          <t>GDT2JN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -924,14 +924,14 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JN</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GDT2JN</t>
+          <t>GDT34Z</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -946,24 +946,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT34Z</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GDT34Z</t>
+          <t>ET1029</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DTA</t>
+          <t>ETA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -973,24 +973,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT34Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ET1029</t>
+          <t>GIE36Z</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ETA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1000,24 +1000,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter godkänd kurs ska studenten kunna:_…</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Z</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GIE26L</t>
+          <t>GIK28T</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1027,24 +1027,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK28T</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GIE26M</t>
+          <t>GIK29B</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1054,24 +1054,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK29B</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GIE26N</t>
+          <t>GIK2Q3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1086,19 +1086,19 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GIE2QS</t>
+          <t>GMA2EY</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1113,19 +1113,19 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2QS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GIE2RF</t>
+          <t>GMD2BH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1135,24 +1135,24 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2RF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GIE36Z</t>
+          <t>GMD2EX</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1162,24 +1162,24 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna:_…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>IE1069</t>
+          <t>GMD2GU</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1189,24 +1189,24 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GIK28T</t>
+          <t>GMD2H2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1216,24 +1216,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK28T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GIK29B</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1243,24 +1243,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK29B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GIK2BD</t>
+          <t>GMD2H4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1270,24 +1270,24 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2BD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GIK2FB</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1297,24 +1297,24 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2FB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GIK2Q3</t>
+          <t>GMD2HE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1324,24 +1324,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GIK2QZ</t>
+          <t>GMD2HF</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1351,24 +1351,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2QZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GIK2UK</t>
+          <t>GMD2HG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1378,24 +1378,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Efter genomförd kurs skall studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2UK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GIK2XJ</t>
+          <t>GMD2HH</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1405,24 +1405,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GIK2XK</t>
+          <t>GMD2HJ</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1437,19 +1437,19 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GIK2YP</t>
+          <t>GMD2HK</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1459,24 +1459,24 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GIK2YR</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1486,24 +1486,24 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GIK32K</t>
+          <t>GMD2MJ</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1513,24 +1513,24 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GIK32L</t>
+          <t>GMD2PA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1540,24 +1540,24 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs ska den studerande…</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GIK32M</t>
+          <t>GMD3GZ</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1567,24 +1567,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GIK32N</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1594,24 +1594,24 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GIK339</t>
+          <t>MD1097</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1621,24 +1621,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK339</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GMA2EY</t>
+          <t>MD1098</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1648,19 +1648,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GMD2BH</t>
+          <t>MD1103</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1680,14 +1680,14 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GMD2EX</t>
+          <t>MD2023</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1707,14 +1707,14 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GMD2GU</t>
+          <t>MD2024</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1734,14 +1734,14 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GMD2H2</t>
+          <t>MD2025</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1761,14 +1761,14 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>MD2026</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1788,19 +1788,19 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GMD2H4</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1810,24 +1810,24 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1837,24 +1837,24 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter godkänd kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GMD2HE</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1864,24 +1864,24 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GMD2HF</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1891,24 +1891,24 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GMD2HG</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1918,24 +1918,24 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GMD2HH</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1945,24 +1945,24 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GMD2HJ</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1972,24 +1972,24 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>GMD2HK</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1999,24 +1999,24 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>GMD2MH</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2026,24 +2026,24 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>GMD2MJ</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2053,24 +2053,24 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>GMD2PA</t>
+          <t>AEG26X</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2080,24 +2080,24 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande…</t>
+          <t>Efter genomgång av kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>GMD3GZ</t>
+          <t>AEG29N</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2107,24 +2107,24 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter godkänd kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG29N</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>AEG2B6</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2134,24 +2134,24 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>MD1097</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2161,24 +2161,24 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>MD1098</t>
+          <t>EG3009</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2188,24 +2188,24 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>MD1103</t>
+          <t>EG3012</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2215,24 +2215,24 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>MD2023</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2242,24 +2242,24 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>MD2024</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2269,24 +2269,24 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter genomgången kurs skall studenten kunna…</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>MD2025</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2296,24 +2296,24 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>MD2026</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2323,24 +2323,24 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2355,19 +2355,19 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>GEG2JP</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2377,24 +2377,24 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GEG39Z</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2404,24 +2404,24 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>GEG3FY</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2431,24 +2431,24 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2463,19 +2463,19 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2485,24 +2485,24 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2517,19 +2517,19 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>GSQ2J4</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2539,24 +2539,24 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna…</t>
+          <t>Efter genomgången kurs ska studenten kunna: ·…</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>GSQ2L8</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2566,24 +2566,24 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter genomgången…</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2593,24 +2593,24 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>AEG26X</t>
+          <t>GSQ2MC</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2620,24 +2620,24 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Efter genomgång av kursen ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>AEG29N</t>
+          <t>GSQ2VY</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2647,24 +2647,24 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Efter godkänd kursen ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>AEG2B6</t>
+          <t>GSQ2WM</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2674,24 +2674,24 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>GSQ33N</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2706,19 +2706,19 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>EG3009</t>
+          <t>GST2CL</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2728,24 +2728,24 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter kursen skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>EG3012</t>
+          <t>ST1013</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2755,24 +2755,24 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter kursen skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>AMI22T</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2782,24 +2782,24 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>AMI23A</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2809,24 +2809,24 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs skall studenten kunna…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>AMI23C</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2836,24 +2836,24 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>AMI23G</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2863,24 +2863,24 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter avslutad kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>AMI23K</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2890,24 +2890,24 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>GEG2JP</t>
+          <t>AMI23L</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2917,24 +2917,24 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs kommer studenten att kunna:…</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>GEG39Z</t>
+          <t>GMI23G</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2944,24 +2944,24 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>GEG3FY</t>
+          <t>GMI24H</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2971,24 +2971,24 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs, ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GMI26H</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2998,24 +2998,24 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>GMI2J3</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3025,24 +3025,24 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>GMI2MD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3052,24 +3052,24 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad utbildning ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>GSQ2J4</t>
+          <t>MI4001</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3079,24 +3079,24 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna: ·…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L8</t>
+          <t>MI4002</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3106,557 +3106,17 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Efter genomgången…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>GSQ2L9</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>GSQ2MC</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>GSQ2VY</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>GSQ2WM</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>GSQ33N</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>GST2CL</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>STA</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Efter kursen skall studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>ST1013</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>STA</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Efter kursen skall studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>AMI22T</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>AMI23A</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>AMI23C</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>AMI23G</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Efter avslutad kursen ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>AMI23K</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>AMI23L</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs kommer studenten att kunna:…</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>GMI23G</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>GMI24H</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>GMI26H</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>GMI2J3</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>GMI2MD</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>Efter avslutad utbildning ska den studerande kunna:…</t>
-        </is>
-      </c>
-      <c r="E117" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>MI4001</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>MI4002</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4002</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E119"/>
+  <autoFilter ref="A1:E99"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -3854,46 +3314,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A102" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A113" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A114" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId236"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans for various subjects, including adjustments to scrape hashes, formatting corrections, and the addition of a new course on cognitive science in education (GMD3K4).
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Frasningskonsistens.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Frasningskonsistens.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Frasningskonsistens" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Frasningskonsistens'!$A$1:$E$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Frasningskonsistens'!$A$1:$E$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -985,12 +985,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GIE36Z</t>
+          <t>GIK28T</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1000,19 +1000,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna:_…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK28T</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GIK28T</t>
+          <t>GIK29B</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1027,19 +1027,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK28T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK29B</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GIK29B</t>
+          <t>GIK2Q3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1059,19 +1059,19 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK29B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GIK2Q3</t>
+          <t>GMA2EY</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1086,19 +1086,19 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GMA2EY</t>
+          <t>GMD2BH</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GMD2BH</t>
+          <t>GMD2EX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1140,14 +1140,14 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GMD2EX</t>
+          <t>GMD2GU</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1167,14 +1167,14 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GMD2GU</t>
+          <t>GMD2H2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1194,14 +1194,14 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GMD2H2</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1221,14 +1221,14 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>GMD2H4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1248,14 +1248,14 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H4</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GMD2H4</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1275,14 +1275,14 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GMD2HE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1302,14 +1302,14 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GMD2HE</t>
+          <t>GMD2HF</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1329,14 +1329,14 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GMD2HF</t>
+          <t>GMD2HG</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1356,14 +1356,14 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GMD2HG</t>
+          <t>GMD2HH</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1383,14 +1383,14 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GMD2HH</t>
+          <t>GMD2HJ</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1410,14 +1410,14 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GMD2HJ</t>
+          <t>GMD2HK</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1437,14 +1437,14 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GMD2HK</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1464,14 +1464,14 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GMD2MH</t>
+          <t>GMD2MJ</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1491,14 +1491,14 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GMD2MJ</t>
+          <t>GMD2PA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande…</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GMD2PA</t>
+          <t>GMD3GZ</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1540,19 +1540,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GMD3GZ</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1572,14 +1572,14 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>MD1097</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1594,19 +1594,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>MD1097</t>
+          <t>MD1098</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1621,19 +1621,19 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MD1098</t>
+          <t>MD1103</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1653,14 +1653,14 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>MD1103</t>
+          <t>MD2023</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1680,14 +1680,14 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>MD2023</t>
+          <t>MD2024</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1707,14 +1707,14 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>MD2024</t>
+          <t>MD2025</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1734,14 +1734,14 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>MD2025</t>
+          <t>MD2026</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1761,19 +1761,19 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MD2026</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1783,19 +1783,19 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1810,19 +1810,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter godkänd kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1837,19 +1837,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1869,14 +1869,14 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1891,19 +1891,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1918,19 +1918,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1945,24 +1945,24 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1972,19 +1972,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1999,19 +1999,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2026,19 +2026,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>AEG26X</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2053,19 +2053,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna…</t>
+          <t>Efter genomgång av kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>AEG26X</t>
+          <t>AEG29N</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2080,19 +2080,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Efter genomgång av kursen ska studenten kunna:…</t>
+          <t>Efter godkänd kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG29N</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AEG29N</t>
+          <t>AEG2B6</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Efter godkänd kursen ska studenten kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AEG2B6</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2134,19 +2134,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>EG3009</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2166,14 +2166,14 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>EG3009</t>
+          <t>EG3012</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2193,14 +2193,14 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>EG3012</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2220,14 +2220,14 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2242,19 +2242,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs skall studenten kunna…</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs skall studenten kunna…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2301,14 +2301,14 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2323,19 +2323,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>GEG2JP</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2350,19 +2350,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GEG2JP</t>
+          <t>GEG39Z</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GEG39Z</t>
+          <t>GEG3FY</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,24 +2404,24 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GEG3FY</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs, ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2463,14 +2463,14 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2490,14 +2490,14 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>GSQ2J4</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2512,19 +2512,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna: ·…</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>GSQ2J4</t>
+          <t>GSQ2L8</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2539,19 +2539,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna: ·…</t>
+          <t>Efter genomgången…</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L8</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2566,19 +2566,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Efter genomgången…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GSQ2MC</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2598,14 +2598,14 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GSQ2MC</t>
+          <t>GSQ2VY</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2620,19 +2620,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GSQ2VY</t>
+          <t>GSQ2WM</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2647,19 +2647,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GSQ2WM</t>
+          <t>GSQ33N</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2679,19 +2679,19 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GSQ33N</t>
+          <t>GST2CL</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2701,19 +2701,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter kursen skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>GST2CL</t>
+          <t>ST1013</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2733,19 +2733,19 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>ST1013</t>
+          <t>AMI22T</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Efter kursen skall studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>AMI22T</t>
+          <t>AMI23A</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2782,19 +2782,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>AMI23A</t>
+          <t>AMI23C</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2809,19 +2809,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>AMI23C</t>
+          <t>AMI23G</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2836,19 +2836,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter avslutad kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>AMI23G</t>
+          <t>AMI23K</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2863,19 +2863,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Efter avslutad kursen ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>AMI23K</t>
+          <t>AMI23L</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2890,19 +2890,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs kommer studenten att kunna:…</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>AMI23L</t>
+          <t>GMI23G</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2917,19 +2917,19 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs kommer studenten att kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>GMI23G</t>
+          <t>GMI24H</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2944,19 +2944,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>GMI24H</t>
+          <t>GMI26H</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2971,19 +2971,19 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>GMI26H</t>
+          <t>GMI2J3</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2998,19 +2998,19 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>GMI2J3</t>
+          <t>GMI2MD</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3025,19 +3025,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad utbildning ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>GMI2MD</t>
+          <t>MI4001</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3052,19 +3052,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Efter avslutad utbildning ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>MI4001</t>
+          <t>MI4002</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3084,39 +3084,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>MI4002</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4002</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E99"/>
+  <autoFilter ref="A1:E98"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -3312,8 +3285,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId196"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans for Kinesiska, Svenska som andraspråk, and various engineering subjects
- Revised Kinesiska course plans to reflect updated course offerings and removed inactive tags.
- Adjusted course count in Svenska som andraspråk MOC and updated course listings, including new additions and removals.
- Added new course plans for "Ledarskap" (GBY3K7), "Basmatematik 2" (BMA229), "Examensarbete i assisterande teknik" (GMT3K5), "Forskningsmetodik för ingenjörer" (GMT3K6), "Ellära" (GEG3K8), and "Styr- och reglerteknik" (GEG3K9) with detailed descriptions and learning outcomes.
- Updated tags and classifications for several courses to ensure consistency and accuracy.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Frasningskonsistens.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Frasningskonsistens.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Frasningskonsistens" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Frasningskonsistens'!$A$1:$E$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Frasningskonsistens'!$A$1:$E$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1066,7 +1066,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GMA2EY</t>
+          <t>BMA229</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1086,19 +1086,19 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA229</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GMD2BH</t>
+          <t>GMA2EY</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GMD2EX</t>
+          <t>GMD2BH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1140,14 +1140,14 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GMD2GU</t>
+          <t>GMD2EX</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1167,14 +1167,14 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GMD2H2</t>
+          <t>GMD2GU</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1194,14 +1194,14 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>GMD2H2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1221,14 +1221,14 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GMD2H4</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1248,14 +1248,14 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GMD2H4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1275,14 +1275,14 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GMD2HE</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1302,14 +1302,14 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GMD2HF</t>
+          <t>GMD2HE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1329,14 +1329,14 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GMD2HG</t>
+          <t>GMD2HF</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1356,14 +1356,14 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GMD2HH</t>
+          <t>GMD2HG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1383,14 +1383,14 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GMD2HJ</t>
+          <t>GMD2HH</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1410,14 +1410,14 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GMD2HK</t>
+          <t>GMD2HJ</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1437,14 +1437,14 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GMD2MH</t>
+          <t>GMD2HK</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1464,14 +1464,14 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GMD2MJ</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1491,14 +1491,14 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GMD2PA</t>
+          <t>GMD2MJ</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GMD3GZ</t>
+          <t>GMD2PA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1540,19 +1540,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande…</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>GMD3GZ</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1572,14 +1572,14 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>MD1097</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1594,19 +1594,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>MD1098</t>
+          <t>MD1097</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1621,19 +1621,19 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MD1103</t>
+          <t>MD1098</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1653,14 +1653,14 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>MD2023</t>
+          <t>MD1103</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1680,14 +1680,14 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>MD2024</t>
+          <t>MD2023</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1707,14 +1707,14 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>MD2025</t>
+          <t>MD2024</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1734,14 +1734,14 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>MD2026</t>
+          <t>MD2025</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1761,19 +1761,19 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MIKR002</t>
+          <t>MD2026</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MIKRODAT</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1783,24 +1783,24 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MIKR002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>MIKR002</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1810,19 +1810,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MIKR002</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1837,19 +1837,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1864,19 +1864,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1896,14 +1896,14 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1918,19 +1918,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1945,19 +1945,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1972,24 +1972,24 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1999,19 +1999,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2026,19 +2026,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2053,19 +2053,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>AEG26X</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2080,19 +2080,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Efter genomgång av kursen ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AEG29N</t>
+          <t>AEG26X</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Efter godkänd kursen ska studenten kunna:…</t>
+          <t>Efter genomgång av kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AEG2B6</t>
+          <t>AEG29N</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2134,19 +2134,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter godkänd kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG29N</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>AEG2B6</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2161,19 +2161,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>EG3009</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2193,14 +2193,14 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>EG3012</t>
+          <t>EG3009</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2220,14 +2220,14 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>EG3012</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2247,14 +2247,14 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs skall studenten kunna…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2296,19 +2296,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs, ska studenten kunna:…</t>
+          <t>Efter genomgången kurs skall studenten kunna…</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2328,14 +2328,14 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2350,19 +2350,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GEG2JP</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GEG39Z</t>
+          <t>GEG2JP</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs skall studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GEG3FY</t>
+          <t>GEG39Z</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2431,24 +2431,24 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Efter godkänd kurs, ska studenten kunna:…</t>
+          <t>Efter godkänd kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GEG3FY</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2458,19 +2458,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter godkänd kurs, ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2490,14 +2490,14 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2517,14 +2517,14 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>GSQ2J4</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2539,19 +2539,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna: ·…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L8</t>
+          <t>GSQ2J4</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2566,19 +2566,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Efter genomgången…</t>
+          <t>Efter genomgången kurs ska studenten kunna: ·…</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GSQ2L8</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2593,19 +2593,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter genomgången…</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GSQ2MC</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2625,14 +2625,14 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GSQ2VY</t>
+          <t>GSQ2MC</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2647,19 +2647,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GSQ2WM</t>
+          <t>GSQ2VY</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2674,19 +2674,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Efter genomgången kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GSQ33N</t>
+          <t>GSQ2WM</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2706,19 +2706,19 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>GST2CL</t>
+          <t>GSQ33N</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2728,19 +2728,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Efter kursen skall studenten kunna:…</t>
+          <t>Efter genomgången kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>ST1013</t>
+          <t>GST2CL</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2760,19 +2760,19 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>AMI22T</t>
+          <t>ST1013</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2782,19 +2782,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter kursen skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>AMI23A</t>
+          <t>AMI22T</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2809,19 +2809,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>AMI23C</t>
+          <t>AMI23A</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2836,19 +2836,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs skall studenten kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>AMI23G</t>
+          <t>AMI23C</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2863,19 +2863,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Efter avslutad kursen ska studenten kunna:…</t>
+          <t>Efter avslutad kurs skall studenten kunna:…</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>AMI23K</t>
+          <t>AMI23G</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2890,19 +2890,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
+          <t>Efter avslutad kursen ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>AMI23L</t>
+          <t>AMI23K</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2917,19 +2917,19 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs kommer studenten att kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>GMI23G</t>
+          <t>AMI23L</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2944,19 +2944,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs kommer studenten att kunna:…</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>GMI24H</t>
+          <t>GMI23G</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2971,19 +2971,19 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>GMI26H</t>
+          <t>GMI24H</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2998,19 +2998,19 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>GMI2J3</t>
+          <t>GMI26H</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3025,19 +3025,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska den studerande kunna…</t>
+          <t>Efter avslutad kurs ska studenten kunna:…</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>GMI2MD</t>
+          <t>GMI2J3</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3052,19 +3052,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Efter avslutad utbildning ska den studerande kunna:…</t>
+          <t>Efter avslutad kurs ska den studerande kunna…</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>MI4001</t>
+          <t>GMI2MD</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3079,44 +3079,71 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Efter avslutad kurs ska studenten kunna…</t>
+          <t>Efter avslutad utbildning ska den studerande kunna:…</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
+          <t>MI4001</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Avviker från referensformen</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Efter avslutad kurs ska studenten kunna…</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
           <t>MI4002</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>XYZ</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Avviker från referensformen</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Avviker från referensformen</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
         <is>
           <t>Efter avslutad kurs ska studenten kunna…</t>
         </is>
       </c>
-      <c r="E99" s="2" t="inlineStr">
+      <c r="E100" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4002</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E99"/>
+  <autoFilter ref="A1:E100"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -3314,6 +3341,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId198"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>